<commit_message>
feat: implement item equipment tests and refactor bot methods
- Add comprehensive item equipment and unequipment test scenarios
- Refactor test_case methods to game_bot class as instance methods
- Add monster spawning, stat setting, and spell management methods to game_bot
- Update skill test files to use new bot method structure
- Add item inactive protocol support and command.lua updates
- Update model definitions and class data table
- Improve test framework with better method organization
</commit_message>
<xml_diff>
--- a/resources/table/class.xlsx
+++ b/resources/table/class.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\git\fb\resources\table\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6099CBCA-7E63-4FBC-9240-3C53D0AF84E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E92D5278-B3C3-418A-8C58-6C30850A98E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{51E714AE-D231-4317-A66B-833316D0EFD8}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{51E714AE-D231-4317-A66B-833316D0EFD8}"/>
   </bookViews>
   <sheets>
     <sheet name="ability" sheetId="1" r:id="rId1"/>
@@ -111,9 +111,6 @@
     <t>진검</t>
   </si>
   <si>
-    <t>귀객</t>
-  </si>
-  <si>
     <t>태성</t>
   </si>
   <si>
@@ -188,6 +185,10 @@
   </si>
   <si>
     <t>NONE</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>귀검</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -640,7 +641,7 @@
         <v>2</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D1" s="3" t="s">
         <v>5</v>
@@ -652,7 +653,7 @@
         <v>7</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="H1" s="3" t="s">
         <v>9</v>
@@ -663,7 +664,7 @@
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>3</v>
@@ -721,7 +722,7 @@
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.3">
@@ -861,7 +862,7 @@
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A10" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B10" s="6"/>
       <c r="C10" s="6"/>
@@ -3439,7 +3440,7 @@
     </row>
     <row r="106" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A106" s="3" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B106" s="6"/>
       <c r="C106" s="6"/>
@@ -6110,7 +6111,7 @@
     </row>
     <row r="202" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A202" s="6" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B202" s="6"/>
       <c r="C202" s="6"/>
@@ -8783,7 +8784,7 @@
     </row>
     <row r="298" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A298" s="6" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B298" s="6"/>
       <c r="C298" s="6"/>
@@ -11476,18 +11477,18 @@
         <v>11</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>3</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
@@ -11503,7 +11504,7 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" s="5" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
@@ -11512,7 +11513,7 @@
         <v>0</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
@@ -11520,7 +11521,7 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
@@ -11565,7 +11566,7 @@
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.3">
@@ -11597,7 +11598,7 @@
         <v>3</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>20</v>
+        <v>42</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.3">
@@ -11605,12 +11606,12 @@
         <v>4</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.3">
@@ -11618,7 +11619,7 @@
         <v>0</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.3">
@@ -11626,7 +11627,7 @@
         <v>1</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.3">
@@ -11634,7 +11635,7 @@
         <v>2</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.3">
@@ -11642,7 +11643,7 @@
         <v>3</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.3">
@@ -11650,12 +11651,12 @@
         <v>4</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A28" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.3">
@@ -11663,7 +11664,7 @@
         <v>0</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.3">
@@ -11671,7 +11672,7 @@
         <v>1</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.3">
@@ -11679,7 +11680,7 @@
         <v>2</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.3">
@@ -11687,7 +11688,7 @@
         <v>3</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="33" spans="2:3" x14ac:dyDescent="0.3">
@@ -11695,7 +11696,7 @@
         <v>4</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
   </sheetData>

</xml_diff>